<commit_message>
clearing columns on template
renaming analysis to data analysis
</commit_message>
<xml_diff>
--- a/SOPs/Lab/general-filtering/templates/filtering-lab-data-sheets.xlsx
+++ b/SOPs/Lab/general-filtering/templates/filtering-lab-data-sheets.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wampleka\Documents\Projects\WWS-standard-methods\SOPs\Lab\general-filtering\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{50407A47-460E-4A7B-A50B-767E89E5F7F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{777A45AA-21E9-49EC-B1CB-AC35032B377D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FILL ME" sheetId="10" r:id="rId1"/>
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="52">
   <si>
     <t>Project</t>
   </si>
@@ -460,6 +460,9 @@
   <si>
     <t>Sample ID Type (choose one)</t>
   </si>
+  <si>
+    <t>For Many Sites Paste Site Names Here</t>
+  </si>
 </sst>
 </file>
 
@@ -801,9 +804,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -831,6 +831,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1263,91 +1264,97 @@
     <col min="1" max="1" width="39.7109375" customWidth="1"/>
     <col min="2" max="2" width="20.42578125" customWidth="1"/>
     <col min="3" max="3" width="24.140625" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" customWidth="1"/>
+    <col min="4" max="4" width="35.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="37" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="37"/>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B1" s="36"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>41</v>
       </c>
       <c r="B3" s="31"/>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D3" s="41" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>42</v>
       </c>
       <c r="B4" s="31"/>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="B5" s="32"/>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B5" s="31" t="str">
+        <f>_xlfn.TEXTJOIN(", ",TRUE,D4:D100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
       <c r="B6" s="31"/>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="33"/>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B7" s="32"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="B8" s="33" t="s">
+      <c r="B8" s="32" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="32" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="38" t="s">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="38"/>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B10" s="37"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="34"/>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B11" s="33"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="B12" s="34"/>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B12" s="33"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="35"/>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B13" s="34"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
         <v>45</v>
       </c>
       <c r="B15" s="14">
-        <f>COUNTA(_xlfn.TEXTSPLIT('FILL ME'!$B$5, ", "))</f>
+        <f>COUNTA(_xlfn.TEXTSPLIT('FILL ME'!#REF!, ", "))</f>
         <v>1</v>
       </c>
     </row>
@@ -1357,12 +1364,12 @@
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="36" t="s">
+      <c r="A18" s="35" t="s">
         <v>38</v>
       </c>
-      <c r="B18" s="36"/>
-      <c r="C18" s="36"/>
-      <c r="D18" s="36"/>
+      <c r="B18" s="35"/>
+      <c r="C18" s="35"/>
+      <c r="D18" s="35"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="30" t="s">
@@ -1373,28 +1380,28 @@
       <c r="D19" s="30"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="36" t="s">
+      <c r="A20" s="35" t="s">
         <v>48</v>
       </c>
-      <c r="B20" s="36"/>
-      <c r="C20" s="36"/>
-      <c r="D20" s="36"/>
+      <c r="B20" s="35"/>
+      <c r="C20" s="35"/>
+      <c r="D20" s="35"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="36" t="s">
+      <c r="A21" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="36"/>
-      <c r="C21" s="36"/>
-      <c r="D21" s="36"/>
+      <c r="B21" s="35"/>
+      <c r="C21" s="35"/>
+      <c r="D21" s="35"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="36" t="s">
+      <c r="A22" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="B22" s="36"/>
-      <c r="C22" s="36"/>
-      <c r="D22" s="36"/>
+      <c r="B22" s="35"/>
+      <c r="C22" s="35"/>
+      <c r="D22" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1479,7 +1486,7 @@
         <v/>
       </c>
       <c r="C2" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D2" s="11" t="str">
@@ -1500,23 +1507,23 @@
       </c>
       <c r="H2" s="3" t="e" cm="1">
         <f t="array" ref="H2">_xlfn.LET(
-    _xlpm.items, _xlfn.TEXTSPLIT('FILL ME'!$B$5, ", "),
+    _xlpm.items, _xlfn.TEXTSPLIT('FILL ME'!#REF!, ", "),
     _xlpm.x, 'FILL ME'!$B$6,
     INDEX(_xlpm.items, ROUNDUP(_xlfn.SEQUENCE(COUNTA(_xlpm.items)*_xlpm.x)/_xlpm.x, 0))
 )</f>
-        <v>#VALUE!</v>
+        <v>#REF!</v>
       </c>
       <c r="I2" s="14" t="e">
         <f>CONCATENATE(H2,"_",TEXT(G2,"00"))</f>
-        <v>#VALUE!</v>
+        <v>#REF!</v>
       </c>
       <c r="J2" s="15" t="e">
         <f>CONCATENATE(C2,"_", H2,"_",D2,"_",TEXT(G2,"00"))</f>
-        <v>#VALUE!</v>
+        <v>#REF!</v>
       </c>
       <c r="K2" s="15" t="e">
         <f>CONCATENATE(C2,"_", H2,"_",TEXT(E2, "yyyymmdd"),"_",TEXT(F2, "hhmm"))</f>
-        <v>#VALUE!</v>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -1529,7 +1536,7 @@
         <v/>
       </c>
       <c r="C3" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D3" s="11" t="str">
@@ -1567,7 +1574,7 @@
         <v/>
       </c>
       <c r="C4" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D4" s="11" t="str">
@@ -1605,7 +1612,7 @@
         <v/>
       </c>
       <c r="C5" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D5" s="11" t="str">
@@ -1643,7 +1650,7 @@
         <v/>
       </c>
       <c r="C6" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D6" s="11" t="str">
@@ -1681,7 +1688,7 @@
         <v/>
       </c>
       <c r="C7" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D7" s="11" t="str">
@@ -1719,7 +1726,7 @@
         <v/>
       </c>
       <c r="C8" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D8" s="11" t="str">
@@ -1757,7 +1764,7 @@
         <v/>
       </c>
       <c r="C9" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D9" s="11" t="str">
@@ -1795,7 +1802,7 @@
         <v/>
       </c>
       <c r="C10" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D10" s="11" t="str">
@@ -1833,7 +1840,7 @@
         <v/>
       </c>
       <c r="C11" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D11" s="11" t="str">
@@ -1871,7 +1878,7 @@
         <v/>
       </c>
       <c r="C12" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D12" s="11" t="str">
@@ -1909,7 +1916,7 @@
         <v/>
       </c>
       <c r="C13" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D13" s="11" t="str">
@@ -1947,7 +1954,7 @@
         <v/>
       </c>
       <c r="C14" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D14" s="11" t="str">
@@ -1985,7 +1992,7 @@
         <v/>
       </c>
       <c r="C15" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D15" s="11" t="str">
@@ -2023,7 +2030,7 @@
         <v/>
       </c>
       <c r="C16" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D16" s="11" t="str">
@@ -2061,7 +2068,7 @@
         <v/>
       </c>
       <c r="C17" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D17" s="11" t="str">
@@ -2099,7 +2106,7 @@
         <v/>
       </c>
       <c r="C18" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D18" s="11" t="str">
@@ -2137,7 +2144,7 @@
         <v/>
       </c>
       <c r="C19" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D19" s="11" t="str">
@@ -2175,7 +2182,7 @@
         <v/>
       </c>
       <c r="C20" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D20" s="11" t="str">
@@ -2213,7 +2220,7 @@
         <v/>
       </c>
       <c r="C21" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D21" s="11" t="str">
@@ -2251,7 +2258,7 @@
         <v/>
       </c>
       <c r="C22" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D22" s="11" t="str">
@@ -2289,7 +2296,7 @@
         <v/>
       </c>
       <c r="C23" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D23" s="11" t="str">
@@ -2327,7 +2334,7 @@
         <v/>
       </c>
       <c r="C24" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D24" s="11" t="str">
@@ -2365,7 +2372,7 @@
         <v/>
       </c>
       <c r="C25" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D25" s="11" t="str">
@@ -2403,7 +2410,7 @@
         <v/>
       </c>
       <c r="C26" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D26" s="11" t="str">
@@ -2441,7 +2448,7 @@
         <v/>
       </c>
       <c r="C27" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D27" s="11" t="str">
@@ -2479,7 +2486,7 @@
         <v/>
       </c>
       <c r="C28" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D28" s="11" t="str">
@@ -2517,7 +2524,7 @@
         <v/>
       </c>
       <c r="C29" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D29" s="11" t="str">
@@ -2555,7 +2562,7 @@
         <v/>
       </c>
       <c r="C30" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D30" s="11" t="str">
@@ -2593,7 +2600,7 @@
         <v/>
       </c>
       <c r="C31" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D31" s="11" t="str">
@@ -2631,7 +2638,7 @@
         <v/>
       </c>
       <c r="C32" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D32" s="11" t="str">
@@ -2669,7 +2676,7 @@
         <v/>
       </c>
       <c r="C33" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D33" s="11" t="str">
@@ -2707,7 +2714,7 @@
         <v/>
       </c>
       <c r="C34" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D34" s="11" t="str">
@@ -2745,7 +2752,7 @@
         <v/>
       </c>
       <c r="C35" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D35" s="11" t="str">
@@ -2783,7 +2790,7 @@
         <v/>
       </c>
       <c r="C36" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D36" s="11" t="str">
@@ -2821,7 +2828,7 @@
         <v/>
       </c>
       <c r="C37" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D37" s="11" t="str">
@@ -2859,7 +2866,7 @@
         <v/>
       </c>
       <c r="C38" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D38" s="11" t="str">
@@ -2897,7 +2904,7 @@
         <v/>
       </c>
       <c r="C39" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D39" s="11" t="str">
@@ -2935,7 +2942,7 @@
         <v/>
       </c>
       <c r="C40" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D40" s="11" t="str">
@@ -2973,7 +2980,7 @@
         <v/>
       </c>
       <c r="C41" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D41" s="11" t="str">
@@ -3011,7 +3018,7 @@
         <v/>
       </c>
       <c r="C42" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D42" s="11" t="str">
@@ -3049,7 +3056,7 @@
         <v/>
       </c>
       <c r="C43" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D43" s="11" t="str">
@@ -3087,7 +3094,7 @@
         <v/>
       </c>
       <c r="C44" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D44" s="11" t="str">
@@ -3125,7 +3132,7 @@
         <v/>
       </c>
       <c r="C45" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D45" s="11" t="str">
@@ -3163,7 +3170,7 @@
         <v/>
       </c>
       <c r="C46" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D46" s="11" t="str">
@@ -3201,7 +3208,7 @@
         <v/>
       </c>
       <c r="C47" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D47" s="11" t="str">
@@ -3239,7 +3246,7 @@
         <v/>
       </c>
       <c r="C48" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D48" s="11" t="str">
@@ -3277,7 +3284,7 @@
         <v/>
       </c>
       <c r="C49" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D49" s="11" t="str">
@@ -3315,7 +3322,7 @@
         <v/>
       </c>
       <c r="C50" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D50" s="11" t="str">
@@ -3354,7 +3361,7 @@
         <v/>
       </c>
       <c r="C51" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D51" s="11" t="str">
@@ -3393,7 +3400,7 @@
         <v/>
       </c>
       <c r="C52" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D52" s="11" t="str">
@@ -3432,7 +3439,7 @@
         <v/>
       </c>
       <c r="C53" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D53" s="11" t="str">
@@ -3471,7 +3478,7 @@
         <v/>
       </c>
       <c r="C54" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D54" s="11" t="str">
@@ -3510,7 +3517,7 @@
         <v/>
       </c>
       <c r="C55" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D55" s="11" t="str">
@@ -3549,7 +3556,7 @@
         <v/>
       </c>
       <c r="C56" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D56" s="11" t="str">
@@ -3588,7 +3595,7 @@
         <v/>
       </c>
       <c r="C57" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D57" s="11" t="str">
@@ -3627,7 +3634,7 @@
         <v/>
       </c>
       <c r="C58" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D58" s="11" t="str">
@@ -3666,7 +3673,7 @@
         <v/>
       </c>
       <c r="C59" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D59" s="11" t="str">
@@ -3705,7 +3712,7 @@
         <v/>
       </c>
       <c r="C60" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D60" s="11" t="str">
@@ -3744,7 +3751,7 @@
         <v/>
       </c>
       <c r="C61" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D61" s="11" t="str">
@@ -3779,7 +3786,7 @@
         <v/>
       </c>
       <c r="C62" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D62" s="11" t="str">
@@ -3814,7 +3821,7 @@
         <v/>
       </c>
       <c r="C63" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D63" s="11" t="str">
@@ -3849,7 +3856,7 @@
         <v/>
       </c>
       <c r="C64" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D64" s="11" t="str">
@@ -3884,7 +3891,7 @@
         <v/>
       </c>
       <c r="C65" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D65" s="11" t="str">
@@ -3919,7 +3926,7 @@
         <v/>
       </c>
       <c r="C66" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D66" s="11" t="str">
@@ -3954,7 +3961,7 @@
         <v/>
       </c>
       <c r="C67" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D67" s="11" t="str">
@@ -3989,7 +3996,7 @@
         <v/>
       </c>
       <c r="C68" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D68" s="11" t="str">
@@ -4024,7 +4031,7 @@
         <v/>
       </c>
       <c r="C69" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D69" s="11" t="str">
@@ -4059,7 +4066,7 @@
         <v/>
       </c>
       <c r="C70" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D70" s="11" t="str">
@@ -4094,7 +4101,7 @@
         <v/>
       </c>
       <c r="C71" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D71" s="11" t="str">
@@ -4129,7 +4136,7 @@
         <v/>
       </c>
       <c r="C72" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D72" s="11" t="str">
@@ -4164,7 +4171,7 @@
         <v/>
       </c>
       <c r="C73" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D73" s="11" t="str">
@@ -4199,7 +4206,7 @@
         <v/>
       </c>
       <c r="C74" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D74" s="11" t="str">
@@ -4234,7 +4241,7 @@
         <v/>
       </c>
       <c r="C75" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D75" s="11" t="str">
@@ -4269,7 +4276,7 @@
         <v/>
       </c>
       <c r="C76" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D76" s="11" t="str">
@@ -4304,7 +4311,7 @@
         <v/>
       </c>
       <c r="C77" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D77" s="11" t="str">
@@ -4339,7 +4346,7 @@
         <v/>
       </c>
       <c r="C78" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D78" s="11" t="str">
@@ -4374,7 +4381,7 @@
         <v/>
       </c>
       <c r="C79" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D79" s="11" t="str">
@@ -4409,7 +4416,7 @@
         <v/>
       </c>
       <c r="C80" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D80" s="11" t="str">
@@ -4444,7 +4451,7 @@
         <v/>
       </c>
       <c r="C81" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D81" s="11" t="str">
@@ -4479,7 +4486,7 @@
         <v/>
       </c>
       <c r="C82" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D82" s="11" t="str">
@@ -4514,7 +4521,7 @@
         <v/>
       </c>
       <c r="C83" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D83" s="11" t="str">
@@ -4549,7 +4556,7 @@
         <v/>
       </c>
       <c r="C84" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D84" s="11" t="str">
@@ -4584,7 +4591,7 @@
         <v/>
       </c>
       <c r="C85" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D85" s="11" t="str">
@@ -4619,7 +4626,7 @@
         <v/>
       </c>
       <c r="C86" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D86" s="11" t="str">
@@ -4654,7 +4661,7 @@
         <v/>
       </c>
       <c r="C87" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D87" s="11" t="str">
@@ -4689,7 +4696,7 @@
         <v/>
       </c>
       <c r="C88" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D88" s="11" t="str">
@@ -4724,7 +4731,7 @@
         <v/>
       </c>
       <c r="C89" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D89" s="11" t="str">
@@ -4759,7 +4766,7 @@
         <v/>
       </c>
       <c r="C90" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D90" s="11" t="str">
@@ -4794,7 +4801,7 @@
         <v/>
       </c>
       <c r="C91" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D91" s="11" t="str">
@@ -4829,7 +4836,7 @@
         <v/>
       </c>
       <c r="C92" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D92" s="11" t="str">
@@ -4864,7 +4871,7 @@
         <v/>
       </c>
       <c r="C93" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D93" s="11" t="str">
@@ -4899,7 +4906,7 @@
         <v/>
       </c>
       <c r="C94" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D94" s="11" t="str">
@@ -4934,7 +4941,7 @@
         <v/>
       </c>
       <c r="C95" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D95" s="11" t="str">
@@ -4969,7 +4976,7 @@
         <v/>
       </c>
       <c r="C96" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D96" s="11" t="str">
@@ -5004,7 +5011,7 @@
         <v/>
       </c>
       <c r="C97" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D97" s="11" t="str">
@@ -5039,7 +5046,7 @@
         <v/>
       </c>
       <c r="C98" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D98" s="11" t="str">
@@ -5074,7 +5081,7 @@
         <v/>
       </c>
       <c r="C99" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D99" s="11" t="str">
@@ -5109,7 +5116,7 @@
         <v/>
       </c>
       <c r="C100" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D100" s="11" t="str">
@@ -5144,7 +5151,7 @@
         <v/>
       </c>
       <c r="C101" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D101" s="11" t="str">
@@ -5179,7 +5186,7 @@
         <v/>
       </c>
       <c r="C102" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D102" s="11" t="str">
@@ -5214,7 +5221,7 @@
         <v/>
       </c>
       <c r="C103" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D103" s="11" t="str">
@@ -5249,7 +5256,7 @@
         <v/>
       </c>
       <c r="C104" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D104" s="11" t="str">
@@ -5284,7 +5291,7 @@
         <v/>
       </c>
       <c r="C105" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D105" s="11" t="str">
@@ -5316,7 +5323,7 @@
         <v/>
       </c>
       <c r="C106" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D106" s="11" t="str">
@@ -5348,7 +5355,7 @@
         <v/>
       </c>
       <c r="C107" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D107" s="11" t="str">
@@ -5380,7 +5387,7 @@
         <v/>
       </c>
       <c r="C108" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D108" s="11" t="str">
@@ -5412,7 +5419,7 @@
         <v/>
       </c>
       <c r="C109" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D109" s="11" t="str">
@@ -5444,7 +5451,7 @@
         <v/>
       </c>
       <c r="C110" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D110" s="11" t="str">
@@ -5476,7 +5483,7 @@
         <v/>
       </c>
       <c r="C111" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D111" s="11" t="str">
@@ -5508,7 +5515,7 @@
         <v/>
       </c>
       <c r="C112" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D112" s="11" t="str">
@@ -5540,7 +5547,7 @@
         <v/>
       </c>
       <c r="C113" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D113" s="11" t="str">
@@ -5572,7 +5579,7 @@
         <v/>
       </c>
       <c r="C114" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D114" s="11" t="str">
@@ -5604,7 +5611,7 @@
         <v/>
       </c>
       <c r="C115" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D115" s="11" t="str">
@@ -5636,7 +5643,7 @@
         <v/>
       </c>
       <c r="C116" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D116" s="11" t="str">
@@ -5668,7 +5675,7 @@
         <v/>
       </c>
       <c r="C117" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D117" s="11" t="str">
@@ -5700,7 +5707,7 @@
         <v/>
       </c>
       <c r="C118" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D118" s="11" t="str">
@@ -5732,7 +5739,7 @@
         <v/>
       </c>
       <c r="C119" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D119" s="11" t="str">
@@ -5764,7 +5771,7 @@
         <v/>
       </c>
       <c r="C120" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D120" s="11" t="str">
@@ -5796,7 +5803,7 @@
         <v/>
       </c>
       <c r="C121" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D121" s="11" t="str">
@@ -5828,7 +5835,7 @@
         <v/>
       </c>
       <c r="C122" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D122" s="11" t="str">
@@ -5860,7 +5867,7 @@
         <v/>
       </c>
       <c r="C123" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D123" s="11" t="str">
@@ -5892,7 +5899,7 @@
         <v/>
       </c>
       <c r="C124" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D124" s="11" t="str">
@@ -5924,7 +5931,7 @@
         <v/>
       </c>
       <c r="C125" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D125" s="11" t="str">
@@ -5956,7 +5963,7 @@
         <v/>
       </c>
       <c r="C126" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D126" s="11" t="str">
@@ -5988,7 +5995,7 @@
         <v/>
       </c>
       <c r="C127" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D127" s="11" t="str">
@@ -6020,7 +6027,7 @@
         <v/>
       </c>
       <c r="C128" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D128" s="11" t="str">
@@ -6052,7 +6059,7 @@
         <v/>
       </c>
       <c r="C129" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D129" s="11" t="str">
@@ -6084,7 +6091,7 @@
         <v/>
       </c>
       <c r="C130" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D130" s="11" t="str">
@@ -6116,7 +6123,7 @@
         <v/>
       </c>
       <c r="C131" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D131" s="11" t="str">
@@ -6148,7 +6155,7 @@
         <v/>
       </c>
       <c r="C132" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D132" s="11" t="str">
@@ -6180,7 +6187,7 @@
         <v/>
       </c>
       <c r="C133" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D133" s="11" t="str">
@@ -6212,7 +6219,7 @@
         <v/>
       </c>
       <c r="C134" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D134" s="11" t="str">
@@ -6244,7 +6251,7 @@
         <v/>
       </c>
       <c r="C135" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D135" s="11" t="str">
@@ -6276,7 +6283,7 @@
         <v/>
       </c>
       <c r="C136" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D136" s="11" t="str">
@@ -6308,7 +6315,7 @@
         <v/>
       </c>
       <c r="C137" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D137" s="11" t="str">
@@ -6340,7 +6347,7 @@
         <v/>
       </c>
       <c r="C138" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D138" s="11" t="str">
@@ -6372,7 +6379,7 @@
         <v/>
       </c>
       <c r="C139" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D139" s="11" t="str">
@@ -6404,7 +6411,7 @@
         <v/>
       </c>
       <c r="C140" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D140" s="11" t="str">
@@ -6436,7 +6443,7 @@
         <v/>
       </c>
       <c r="C141" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D141" s="11" t="str">
@@ -6468,7 +6475,7 @@
         <v/>
       </c>
       <c r="C142" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D142" s="11" t="str">
@@ -6500,7 +6507,7 @@
         <v/>
       </c>
       <c r="C143" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D143" s="11" t="str">
@@ -6532,7 +6539,7 @@
         <v/>
       </c>
       <c r="C144" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D144" s="11" t="str">
@@ -6564,7 +6571,7 @@
         <v/>
       </c>
       <c r="C145" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D145" s="11" t="str">
@@ -6596,7 +6603,7 @@
         <v/>
       </c>
       <c r="C146" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D146" s="11" t="str">
@@ -6628,7 +6635,7 @@
         <v/>
       </c>
       <c r="C147" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D147" s="11" t="str">
@@ -6660,7 +6667,7 @@
         <v/>
       </c>
       <c r="C148" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D148" s="11" t="str">
@@ -6692,7 +6699,7 @@
         <v/>
       </c>
       <c r="C149" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D149" s="11" t="str">
@@ -6724,7 +6731,7 @@
         <v/>
       </c>
       <c r="C150" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D150" s="11" t="str">
@@ -6756,7 +6763,7 @@
         <v/>
       </c>
       <c r="C151" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D151" s="11" t="str">
@@ -6788,7 +6795,7 @@
         <v/>
       </c>
       <c r="C152" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D152" s="11" t="str">
@@ -6820,7 +6827,7 @@
         <v/>
       </c>
       <c r="C153" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D153" s="11" t="str">
@@ -6852,7 +6859,7 @@
         <v/>
       </c>
       <c r="C154" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D154" s="11" t="str">
@@ -6884,7 +6891,7 @@
         <v/>
       </c>
       <c r="C155" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D155" s="11" t="str">
@@ -6916,7 +6923,7 @@
         <v/>
       </c>
       <c r="C156" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D156" s="11" t="str">
@@ -6948,7 +6955,7 @@
         <v/>
       </c>
       <c r="C157" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D157" s="11" t="str">
@@ -6980,7 +6987,7 @@
         <v/>
       </c>
       <c r="C158" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D158" s="11" t="str">
@@ -7012,7 +7019,7 @@
         <v/>
       </c>
       <c r="C159" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D159" s="11" t="str">
@@ -7044,7 +7051,7 @@
         <v/>
       </c>
       <c r="C160" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D160" s="11" t="str">
@@ -7076,7 +7083,7 @@
         <v/>
       </c>
       <c r="C161" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D161" s="11" t="str">
@@ -7108,7 +7115,7 @@
         <v/>
       </c>
       <c r="C162" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D162" s="11" t="str">
@@ -7140,7 +7147,7 @@
         <v/>
       </c>
       <c r="C163" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D163" s="11" t="str">
@@ -7172,7 +7179,7 @@
         <v/>
       </c>
       <c r="C164" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D164" s="11" t="str">
@@ -7204,7 +7211,7 @@
         <v/>
       </c>
       <c r="C165" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D165" s="11" t="str">
@@ -7236,7 +7243,7 @@
         <v/>
       </c>
       <c r="C166" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D166" s="11" t="str">
@@ -7268,7 +7275,7 @@
         <v/>
       </c>
       <c r="C167" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D167" s="11" t="str">
@@ -7300,7 +7307,7 @@
         <v/>
       </c>
       <c r="C168" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D168" s="11" t="str">
@@ -7332,7 +7339,7 @@
         <v/>
       </c>
       <c r="C169" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D169" s="11" t="str">
@@ -7364,7 +7371,7 @@
         <v/>
       </c>
       <c r="C170" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D170" s="11" t="str">
@@ -7396,7 +7403,7 @@
         <v/>
       </c>
       <c r="C171" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D171" s="11" t="str">
@@ -7428,7 +7435,7 @@
         <v/>
       </c>
       <c r="C172" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D172" s="11" t="str">
@@ -7460,7 +7467,7 @@
         <v/>
       </c>
       <c r="C173" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D173" s="11" t="str">
@@ -7492,7 +7499,7 @@
         <v/>
       </c>
       <c r="C174" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D174" s="11" t="str">
@@ -7524,7 +7531,7 @@
         <v/>
       </c>
       <c r="C175" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D175" s="11" t="str">
@@ -7556,7 +7563,7 @@
         <v/>
       </c>
       <c r="C176" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D176" s="11" t="str">
@@ -7588,7 +7595,7 @@
         <v/>
       </c>
       <c r="C177" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D177" s="11" t="str">
@@ -7620,7 +7627,7 @@
         <v/>
       </c>
       <c r="C178" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D178" s="11" t="str">
@@ -7652,7 +7659,7 @@
         <v/>
       </c>
       <c r="C179" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D179" s="11" t="str">
@@ -7684,7 +7691,7 @@
         <v/>
       </c>
       <c r="C180" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D180" s="11" t="str">
@@ -7716,7 +7723,7 @@
         <v/>
       </c>
       <c r="C181" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D181" s="11" t="str">
@@ -7748,7 +7755,7 @@
         <v/>
       </c>
       <c r="C182" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D182" s="11" t="str">
@@ -7780,7 +7787,7 @@
         <v/>
       </c>
       <c r="C183" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D183" s="11" t="str">
@@ -7812,7 +7819,7 @@
         <v/>
       </c>
       <c r="C184" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D184" s="11" t="str">
@@ -7844,7 +7851,7 @@
         <v/>
       </c>
       <c r="C185" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D185" s="11" t="str">
@@ -7876,7 +7883,7 @@
         <v/>
       </c>
       <c r="C186" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D186" s="11" t="str">
@@ -7908,7 +7915,7 @@
         <v/>
       </c>
       <c r="C187" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D187" s="11" t="str">
@@ -7940,7 +7947,7 @@
         <v/>
       </c>
       <c r="C188" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D188" s="11" t="str">
@@ -7972,7 +7979,7 @@
         <v/>
       </c>
       <c r="C189" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D189" s="11" t="str">
@@ -8004,7 +8011,7 @@
         <v/>
       </c>
       <c r="C190" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D190" s="11" t="str">
@@ -8036,7 +8043,7 @@
         <v/>
       </c>
       <c r="C191" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D191" s="11" t="str">
@@ -8068,7 +8075,7 @@
         <v/>
       </c>
       <c r="C192" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D192" s="11" t="str">
@@ -8100,7 +8107,7 @@
         <v/>
       </c>
       <c r="C193" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D193" s="11" t="str">
@@ -8132,7 +8139,7 @@
         <v/>
       </c>
       <c r="C194" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D194" s="11" t="str">
@@ -8164,7 +8171,7 @@
         <v/>
       </c>
       <c r="C195" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D195" s="11" t="str">
@@ -8196,7 +8203,7 @@
         <v/>
       </c>
       <c r="C196" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D196" s="11" t="str">
@@ -8228,7 +8235,7 @@
         <v/>
       </c>
       <c r="C197" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D197" s="11" t="str">
@@ -8260,7 +8267,7 @@
         <v/>
       </c>
       <c r="C198" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D198" s="11" t="str">
@@ -8292,7 +8299,7 @@
         <v/>
       </c>
       <c r="C199" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D199" s="11" t="str">
@@ -8324,7 +8331,7 @@
         <v/>
       </c>
       <c r="C200" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D200" s="11" t="str">
@@ -8356,7 +8363,7 @@
         <v/>
       </c>
       <c r="C201" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D201" s="11" t="str">
@@ -8388,7 +8395,7 @@
         <v/>
       </c>
       <c r="C202" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D202" s="11" t="str">
@@ -8420,7 +8427,7 @@
         <v/>
       </c>
       <c r="C203" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D203" s="11" t="str">
@@ -8452,7 +8459,7 @@
         <v/>
       </c>
       <c r="C204" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D204" s="11" t="str">
@@ -8484,7 +8491,7 @@
         <v/>
       </c>
       <c r="C205" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D205" s="11" t="str">
@@ -8516,7 +8523,7 @@
         <v/>
       </c>
       <c r="C206" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D206" s="11" t="str">
@@ -8548,7 +8555,7 @@
         <v/>
       </c>
       <c r="C207" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D207" s="11" t="str">
@@ -8580,7 +8587,7 @@
         <v/>
       </c>
       <c r="C208" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D208" s="11" t="str">
@@ -8612,7 +8619,7 @@
         <v/>
       </c>
       <c r="C209" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D209" s="11" t="str">
@@ -8644,7 +8651,7 @@
         <v/>
       </c>
       <c r="C210" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D210" s="11" t="str">
@@ -8676,7 +8683,7 @@
         <v/>
       </c>
       <c r="C211" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D211" s="11" t="str">
@@ -8708,7 +8715,7 @@
         <v/>
       </c>
       <c r="C212" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D212" s="11" t="str">
@@ -8740,7 +8747,7 @@
         <v/>
       </c>
       <c r="C213" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D213" s="11" t="str">
@@ -8772,7 +8779,7 @@
         <v/>
       </c>
       <c r="C214" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D214" s="11" t="str">
@@ -8804,7 +8811,7 @@
         <v/>
       </c>
       <c r="C215" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D215" s="11" t="str">
@@ -8836,7 +8843,7 @@
         <v/>
       </c>
       <c r="C216" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D216" s="11" t="str">
@@ -8868,7 +8875,7 @@
         <v/>
       </c>
       <c r="C217" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D217" s="11" t="str">
@@ -8900,7 +8907,7 @@
         <v/>
       </c>
       <c r="C218" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D218" s="11" t="str">
@@ -8932,7 +8939,7 @@
         <v/>
       </c>
       <c r="C219" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D219" s="11" t="str">
@@ -8964,7 +8971,7 @@
         <v/>
       </c>
       <c r="C220" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D220" s="11" t="str">
@@ -8996,7 +9003,7 @@
         <v/>
       </c>
       <c r="C221" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D221" s="11" t="str">
@@ -9028,7 +9035,7 @@
         <v/>
       </c>
       <c r="C222" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D222" s="11" t="str">
@@ -9060,7 +9067,7 @@
         <v/>
       </c>
       <c r="C223" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D223" s="11" t="str">
@@ -9092,7 +9099,7 @@
         <v/>
       </c>
       <c r="C224" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D224" s="11" t="str">
@@ -9124,7 +9131,7 @@
         <v/>
       </c>
       <c r="C225" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D225" s="11" t="str">
@@ -9156,7 +9163,7 @@
         <v/>
       </c>
       <c r="C226" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D226" s="11" t="str">
@@ -9188,7 +9195,7 @@
         <v/>
       </c>
       <c r="C227" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D227" s="11" t="str">
@@ -9220,7 +9227,7 @@
         <v/>
       </c>
       <c r="C228" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D228" s="11" t="str">
@@ -9252,7 +9259,7 @@
         <v/>
       </c>
       <c r="C229" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D229" s="11" t="str">
@@ -9284,7 +9291,7 @@
         <v/>
       </c>
       <c r="C230" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D230" s="11" t="str">
@@ -9316,7 +9323,7 @@
         <v/>
       </c>
       <c r="C231" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D231" s="11" t="str">
@@ -9348,7 +9355,7 @@
         <v/>
       </c>
       <c r="C232" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D232" s="11" t="str">
@@ -9380,7 +9387,7 @@
         <v/>
       </c>
       <c r="C233" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D233" s="11" t="str">
@@ -9412,7 +9419,7 @@
         <v/>
       </c>
       <c r="C234" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D234" s="11" t="str">
@@ -9444,7 +9451,7 @@
         <v/>
       </c>
       <c r="C235" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D235" s="11" t="str">
@@ -9476,7 +9483,7 @@
         <v/>
       </c>
       <c r="C236" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D236" s="11" t="str">
@@ -9508,7 +9515,7 @@
         <v/>
       </c>
       <c r="C237" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D237" s="11" t="str">
@@ -9540,7 +9547,7 @@
         <v/>
       </c>
       <c r="C238" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D238" s="11" t="str">
@@ -9572,7 +9579,7 @@
         <v/>
       </c>
       <c r="C239" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D239" s="11" t="str">
@@ -9604,7 +9611,7 @@
         <v/>
       </c>
       <c r="C240" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D240" s="11" t="str">
@@ -9636,7 +9643,7 @@
         <v/>
       </c>
       <c r="C241" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D241" s="11" t="str">
@@ -9668,7 +9675,7 @@
         <v/>
       </c>
       <c r="C242" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D242" s="11" t="str">
@@ -9700,7 +9707,7 @@
         <v/>
       </c>
       <c r="C243" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D243" s="11" t="str">
@@ -9732,7 +9739,7 @@
         <v/>
       </c>
       <c r="C244" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D244" s="11" t="str">
@@ -9764,7 +9771,7 @@
         <v/>
       </c>
       <c r="C245" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D245" s="11" t="str">
@@ -9796,7 +9803,7 @@
         <v/>
       </c>
       <c r="C246" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D246" s="11" t="str">
@@ -9828,7 +9835,7 @@
         <v/>
       </c>
       <c r="C247" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D247" s="11" t="str">
@@ -9860,7 +9867,7 @@
         <v/>
       </c>
       <c r="C248" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D248" s="11" t="str">
@@ -9892,7 +9899,7 @@
         <v/>
       </c>
       <c r="C249" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D249" s="11" t="str">
@@ -9924,7 +9931,7 @@
         <v/>
       </c>
       <c r="C250" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D250" s="11" t="str">
@@ -9956,7 +9963,7 @@
         <v/>
       </c>
       <c r="C251" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D251" s="11" t="str">
@@ -9988,7 +9995,7 @@
         <v/>
       </c>
       <c r="C252" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D252" s="11" t="str">
@@ -10020,7 +10027,7 @@
         <v/>
       </c>
       <c r="C253" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D253" s="11" t="str">
@@ -10052,7 +10059,7 @@
         <v/>
       </c>
       <c r="C254" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D254" s="11" t="str">
@@ -10084,7 +10091,7 @@
         <v/>
       </c>
       <c r="C255" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D255" s="11" t="str">
@@ -10116,7 +10123,7 @@
         <v/>
       </c>
       <c r="C256" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D256" s="11" t="str">
@@ -10148,7 +10155,7 @@
         <v/>
       </c>
       <c r="C257" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D257" s="11" t="str">
@@ -10180,7 +10187,7 @@
         <v/>
       </c>
       <c r="C258" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D258" s="11" t="str">
@@ -10212,7 +10219,7 @@
         <v/>
       </c>
       <c r="C259" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D259" s="11" t="str">
@@ -10244,7 +10251,7 @@
         <v/>
       </c>
       <c r="C260" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D260" s="11" t="str">
@@ -10276,7 +10283,7 @@
         <v/>
       </c>
       <c r="C261" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D261" s="11" t="str">
@@ -10308,7 +10315,7 @@
         <v/>
       </c>
       <c r="C262" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D262" s="11" t="str">
@@ -10340,7 +10347,7 @@
         <v/>
       </c>
       <c r="C263" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D263" s="11" t="str">
@@ -10372,7 +10379,7 @@
         <v/>
       </c>
       <c r="C264" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D264" s="11" t="str">
@@ -10404,7 +10411,7 @@
         <v/>
       </c>
       <c r="C265" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D265" s="11" t="str">
@@ -10436,7 +10443,7 @@
         <v/>
       </c>
       <c r="C266" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D266" s="11" t="str">
@@ -10468,7 +10475,7 @@
         <v/>
       </c>
       <c r="C267" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D267" s="11" t="str">
@@ -10500,7 +10507,7 @@
         <v/>
       </c>
       <c r="C268" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D268" s="11" t="str">
@@ -10532,7 +10539,7 @@
         <v/>
       </c>
       <c r="C269" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D269" s="11" t="str">
@@ -10564,7 +10571,7 @@
         <v/>
       </c>
       <c r="C270" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D270" s="11" t="str">
@@ -10596,7 +10603,7 @@
         <v/>
       </c>
       <c r="C271" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D271" s="11" t="str">
@@ -10628,7 +10635,7 @@
         <v/>
       </c>
       <c r="C272" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D272" s="11" t="str">
@@ -10660,7 +10667,7 @@
         <v/>
       </c>
       <c r="C273" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D273" s="11" t="str">
@@ -10692,7 +10699,7 @@
         <v/>
       </c>
       <c r="C274" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D274" s="11" t="str">
@@ -10724,7 +10731,7 @@
         <v/>
       </c>
       <c r="C275" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D275" s="11" t="str">
@@ -10756,7 +10763,7 @@
         <v/>
       </c>
       <c r="C276" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D276" s="11" t="str">
@@ -10788,7 +10795,7 @@
         <v/>
       </c>
       <c r="C277" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D277" s="11" t="str">
@@ -10820,7 +10827,7 @@
         <v/>
       </c>
       <c r="C278" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D278" s="11" t="str">
@@ -10852,7 +10859,7 @@
         <v/>
       </c>
       <c r="C279" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D279" s="11" t="str">
@@ -10884,7 +10891,7 @@
         <v/>
       </c>
       <c r="C280" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D280" s="11" t="str">
@@ -10916,7 +10923,7 @@
         <v/>
       </c>
       <c r="C281" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D281" s="11" t="str">
@@ -10948,7 +10955,7 @@
         <v/>
       </c>
       <c r="C282" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D282" s="11" t="str">
@@ -10980,7 +10987,7 @@
         <v/>
       </c>
       <c r="C283" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D283" s="11" t="str">
@@ -11012,7 +11019,7 @@
         <v/>
       </c>
       <c r="C284" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D284" s="11" t="str">
@@ -11044,7 +11051,7 @@
         <v/>
       </c>
       <c r="C285" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D285" s="11" t="str">
@@ -11076,7 +11083,7 @@
         <v/>
       </c>
       <c r="C286" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D286" s="11" t="str">
@@ -11108,7 +11115,7 @@
         <v/>
       </c>
       <c r="C287" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D287" s="11" t="str">
@@ -11140,7 +11147,7 @@
         <v/>
       </c>
       <c r="C288" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D288" s="11" t="str">
@@ -11172,7 +11179,7 @@
         <v/>
       </c>
       <c r="C289" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D289" s="11" t="str">
@@ -11204,7 +11211,7 @@
         <v/>
       </c>
       <c r="C290" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D290" s="11" t="str">
@@ -11236,7 +11243,7 @@
         <v/>
       </c>
       <c r="C291" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D291" s="11" t="str">
@@ -11268,7 +11275,7 @@
         <v/>
       </c>
       <c r="C292" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D292" s="11" t="str">
@@ -11300,7 +11307,7 @@
         <v/>
       </c>
       <c r="C293" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D293" s="11" t="str">
@@ -11332,7 +11339,7 @@
         <v/>
       </c>
       <c r="C294" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D294" s="11" t="str">
@@ -11364,7 +11371,7 @@
         <v/>
       </c>
       <c r="C295" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D295" s="11" t="str">
@@ -11396,7 +11403,7 @@
         <v/>
       </c>
       <c r="C296" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D296" s="11" t="str">
@@ -11428,7 +11435,7 @@
         <v/>
       </c>
       <c r="C297" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D297" s="11" t="str">
@@ -11460,7 +11467,7 @@
         <v/>
       </c>
       <c r="C298" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D298" s="11" t="str">
@@ -11492,7 +11499,7 @@
         <v/>
       </c>
       <c r="C299" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D299" s="11" t="str">
@@ -11524,7 +11531,7 @@
         <v/>
       </c>
       <c r="C300" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D300" s="11" t="str">
@@ -11556,7 +11563,7 @@
         <v/>
       </c>
       <c r="C301" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D301" s="11" t="str">
@@ -11588,7 +11595,7 @@
         <v/>
       </c>
       <c r="C302" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D302" s="11" t="str">
@@ -11620,7 +11627,7 @@
         <v/>
       </c>
       <c r="C303" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D303" s="11" t="str">
@@ -11652,7 +11659,7 @@
         <v/>
       </c>
       <c r="C304" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D304" s="11" t="str">
@@ -11684,7 +11691,7 @@
         <v/>
       </c>
       <c r="C305" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D305" s="11" t="str">
@@ -11716,7 +11723,7 @@
         <v/>
       </c>
       <c r="C306" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D306" s="11" t="str">
@@ -11748,7 +11755,7 @@
         <v/>
       </c>
       <c r="C307" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D307" s="11" t="str">
@@ -11780,7 +11787,7 @@
         <v/>
       </c>
       <c r="C308" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D308" s="11" t="str">
@@ -11812,7 +11819,7 @@
         <v/>
       </c>
       <c r="C309" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D309" s="11" t="str">
@@ -11844,7 +11851,7 @@
         <v/>
       </c>
       <c r="C310" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D310" s="11" t="str">
@@ -11876,7 +11883,7 @@
         <v/>
       </c>
       <c r="C311" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D311" s="11" t="str">
@@ -11908,7 +11915,7 @@
         <v/>
       </c>
       <c r="C312" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D312" s="11" t="str">
@@ -11940,7 +11947,7 @@
         <v/>
       </c>
       <c r="C313" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D313" s="11" t="str">
@@ -11972,7 +11979,7 @@
         <v/>
       </c>
       <c r="C314" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D314" s="11" t="str">
@@ -12004,7 +12011,7 @@
         <v/>
       </c>
       <c r="C315" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D315" s="11" t="str">
@@ -12036,7 +12043,7 @@
         <v/>
       </c>
       <c r="C316" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D316" s="11" t="str">
@@ -12068,7 +12075,7 @@
         <v/>
       </c>
       <c r="C317" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D317" s="11" t="str">
@@ -12100,7 +12107,7 @@
         <v/>
       </c>
       <c r="C318" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D318" s="11" t="str">
@@ -12132,7 +12139,7 @@
         <v/>
       </c>
       <c r="C319" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D319" s="11" t="str">
@@ -12164,7 +12171,7 @@
         <v/>
       </c>
       <c r="C320" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D320" s="11" t="str">
@@ -12196,7 +12203,7 @@
         <v/>
       </c>
       <c r="C321" t="str">
-        <f>IF('FILL ME'!$B$4 = "", "", 'FILL ME'!$B$4)</f>
+        <f>IF('FILL ME'!$B$5 = "", "", 'FILL ME'!$B$5)</f>
         <v/>
       </c>
       <c r="D321" s="11" t="str">
@@ -14117,11 +14124,11 @@
       <c r="A1" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="39" t="s">
+      <c r="B1" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="C1" s="40"/>
-      <c r="D1" s="41" t="s">
+      <c r="C1" s="39"/>
+      <c r="D1" s="40" t="s">
         <v>3</v>
       </c>
     </row>
@@ -14135,7 +14142,7 @@
       <c r="C2" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="D2" s="41"/>
+      <c r="D2" s="40"/>
     </row>
     <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="e" cm="1" vm="2">
@@ -14758,11 +14765,11 @@
       <c r="A1" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="39" t="s">
+      <c r="B1" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="40"/>
-      <c r="D1" s="41" t="s">
+      <c r="C1" s="39"/>
+      <c r="D1" s="40" t="s">
         <v>3</v>
       </c>
     </row>
@@ -14776,7 +14783,7 @@
       <c r="C2" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="D2" s="41"/>
+      <c r="D2" s="40"/>
     </row>
     <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="e" cm="1" vm="2">

</xml_diff>